<commit_message>
feat(F-NAR-019): TREE-DIF-054 passe agent après apply
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-DIF-054.xlsx
+++ b/stories/arbres/TREE-DIF-054.xlsx
@@ -2908,17 +2908,17 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>La lune rentre dans le poing, un petit clic. Il marche ! Sur le mur du buffet, tout droit. Bravo. Le drap blanc tient le carton, droit. Une miette sèche sur le bois. Le buffet redevient calme, autour des assiettes. Le savon de la cuisine sent, tiède.</t>
+          <t>La lune rentre dans le poing, un petit clic. Il marche ! Sur le mur du buffet, tout droit. Regarde ses oreilles, droites. Le drap blanc tient le carton, droit. Une miette sèche sur le bois. Le buffet se tait autour des assiettes. Le savon de la cuisine sent, tiède.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La lune rentre dans le poing, un petit clic. Il marche ! Sur le mur du buffet, tout droit. Bravo. Le drap blanc tient le carton, droit. Une miette sèche sur le bois. Le buffet redevient calme, autour des assiettes. Le savon de la cuisine sent, tiède.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La lune rentre dans le poing, un petit clic. Il marche ! Sur le mur du buffet, tout droit. Regarde ses oreilles, droites. Le drap blanc tient le carton, droit. Une miette sèche sur le bois. Le buffet se tait autour des assiettes. Le savon de la cuisine sent, tiède.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La lune rentre dans le poing, un petit clic. Il marche ! Sur le mur du buffet, tout droit. Bravo. Le drap blanc tient le carton, droit. Une miette sèche sur le bois. Le buffet redevient calme, autour des assiettes. Le savon de la cuisine sent, tiède.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La lune rentre dans le poing, un petit clic. Il marche ! Sur le mur du buffet, tout droit. Regarde ses oreilles, droites. Le drap blanc tient le carton, droit. Une miette sèche sur le bois. Le buffet se tait autour des assiettes. Le savon de la cuisine sent, tiède.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr"/>
@@ -3059,10 +3059,10 @@
           <t>narrateur|La lune rentre dans le poing, un petit clic.
 enfant-f|Il marche !
 papa|Sur le mur du buffet, tout droit.
-maman|Bravo.
+maman|Regarde ses oreilles, droites.
 narrateur|Le drap blanc tient le carton, droit.
 narrateur|Une miette sèche sur le bois.
-narrateur|Le buffet redevient calme, autour des assiettes.
+narrateur|Le buffet se tait autour des assiettes.
 narrateur|Le savon de la cuisine sent, tiède.</t>
         </is>
       </c>
@@ -3279,17 +3279,17 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Le loup part, gris, entre les ombres des assiettes. J'ai posé la serviette, d'abord. Puis le mot est venu. Venez, le mur est prêt. Le drap blanc tient le carton, droit. Victorina pose le carton contre l'épaule. Une assiette tinte, puis se tait. Le couloir laisse un rai, mince.</t>
+          <t>Le loup part, gris, entre les ombres des assiettes. J'ai posé la serviette, d'abord. Puis le mot est venu. Venez, le mur est prêt. Le drap blanc tient le carton, droit. Victorina pose le carton contre l'épaule. Une assiette tinte, puis se tait. Un rai mince coupe le linge, puis s'arrête.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le &lt;emphasis level="moderate"&gt;loup&lt;/emphasis&gt; part, gris, entre les ombres des assiettes. J'ai posé la serviette, d'abord. Puis le mot est venu. Venez, le mur est prêt. Le drap blanc tient le carton, droit. Victorina pose le carton contre l'épaule. Une assiette tinte, puis se tait. Le couloir laisse un rai, mince.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le &lt;emphasis level="moderate"&gt;loup&lt;/emphasis&gt; part, gris, entre les ombres des assiettes. J'ai posé la serviette, d'abord. Puis le mot est venu. Venez, le mur est prêt. Le drap blanc tient le carton, droit. Victorina pose le carton contre l'épaule. Une assiette tinte, puis se tait. Un rai mince coupe le linge, puis s'arrête.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le &lt;emphasis&gt;loup&lt;/emphasis&gt; part, gris, entre les ombres des assiettes. J'ai posé la serviette, d'abord. Puis le mot est venu. Venez, le mur est prêt. Le drap blanc tient le carton, droit. Victorina pose le carton contre l'épaule. Une assiette tinte, puis se tait. Le couloir laisse un rai, mince.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le &lt;emphasis&gt;loup&lt;/emphasis&gt; part, gris, entre les ombres des assiettes. J'ai posé la serviette, d'abord. Puis le mot est venu. Venez, le mur est prêt. Le drap blanc tient le carton, droit. Victorina pose le carton contre l'épaule. Une assiette tinte, puis se tait. Un rai mince coupe le linge, puis s'arrête.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr"/>
@@ -3434,7 +3434,7 @@
 narrateur|Le drap blanc tient le carton, droit.
 narrateur|Victorina pose le carton contre l'épaule.
 narrateur|Une assiette tinte, puis se tait.
-narrateur|Le couloir laisse un rai, mince.</t>
+narrateur|Un rai mince coupe le linge, puis s'arrête.</t>
         </is>
       </c>
       <c r="AX13" t="inlineStr">
@@ -3650,17 +3650,17 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Contre la chaise, le loup tient. On s'est assises, papa. Le haut gardera son ombre. Tiens bien le carton. Le drap blanc tient le carton, droit. Victorina tapote le bois, léger. Une poussière s'envole, puis retombe. Une horloge tape, puis le buffet se tait.</t>
+          <t>Contre la chaise, le loup tient. On s'est assises, papa. Le haut gardera son ombre. Tiens bien le carton. Le drap blanc tient le carton, droit. Victorina tapote le bois, léger. Une poussière s'envole, puis retombe. L'horloge tape une fois, le buffet se tait.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Contre la chaise, le &lt;emphasis level="moderate"&gt;loup&lt;/emphasis&gt; tient. On s'est assises, papa. Le haut gardera son ombre. Tiens bien le carton. Le drap blanc tient le carton, droit. Victorina tapote le bois, léger. Une poussière s'envole, puis retombe. Une horloge tape, puis le buffet se tait.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Contre la chaise, le &lt;emphasis level="moderate"&gt;loup&lt;/emphasis&gt; tient. On s'est assises, papa. Le haut gardera son ombre. Tiens bien le carton. Le drap blanc tient le carton, droit. Victorina tapote le bois, léger. Une poussière s'envole, puis retombe. L'horloge tape une fois, le buffet se tait.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Contre la chaise, le &lt;emphasis&gt;loup&lt;/emphasis&gt; tient. On s'est assises, papa. Le haut gardera son ombre. Tiens bien le carton. Le drap blanc tient le carton, droit. Victorina tapote le bois, léger. Une poussière s'envole, puis retombe. Une horloge tape, puis le buffet se tait.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Contre la chaise, le &lt;emphasis&gt;loup&lt;/emphasis&gt; tient. On s'est assises, papa. Le haut gardera son ombre. Tiens bien le carton. Le drap blanc tient le carton, droit. Victorina tapote le bois, léger. Une poussière s'envole, puis retombe. L'horloge tape une fois, le buffet se tait.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr"/>
@@ -3805,7 +3805,7 @@
 narrateur|Le drap blanc tient le carton, droit.
 narrateur|Victorina tapote le bois, léger.
 narrateur|Une poussière s'envole, puis retombe.
-narrateur|Une horloge tape, puis le buffet se tait.</t>
+narrateur|L'horloge tape une fois, le buffet se tait.</t>
         </is>
       </c>
       <c r="AX15" t="inlineStr">
@@ -4593,17 +4593,17 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Tout bas, ici. Tout près des oreilles. L'écho devient un peu plus loin. Derrière. Victorina attend, les lèvres fermées. Derrière la boîte. Le drap blanc reste contre la jambe, sage. On a chuchoté ensemble. La suite a eu sa place.</t>
+          <t>Tout bas, ici. Tout près des oreilles. L'écho devient un peu plus loin. Derrière. Victorina attend, les lèvres fermées. Derrière la boîte. Le drap blanc reste contre la jambe, sage. On a chuchoté ensemble. On l'entend, maintenant.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Tout bas, ici. Tout près des oreilles. L'écho devient un peu plus loin. Derrière. Victorina attend, les lèvres fermées. Derrière la boîte. Le drap blanc reste contre la jambe, sage. On a chuchoté ensemble. La suite a eu sa place.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Tout bas, ici. Tout près des oreilles. L'écho devient un peu plus loin. Derrière. Victorina attend, les lèvres fermées. Derrière la boîte. Le drap blanc reste contre la jambe, sage. On a chuchoté ensemble. On l'entend, maintenant.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Tout bas, ici. Tout près des oreilles. L'écho devient un peu plus loin. Derrière. Victorina attend, les lèvres fermées. Derrière la boîte. Le drap blanc reste contre la jambe, sage. On a chuchoté ensemble. La suite a eu sa place. [pause]</t>
+          <t>Tout bas, ici. Tout près des oreilles. L'écho devient un peu plus loin. Derrière. Victorina attend, les lèvres fermées. Derrière la boîte. Le drap blanc reste contre la jambe, sage. On a chuchoté ensemble. On l'entend, maintenant. [pause]</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr"/>
@@ -4745,7 +4745,7 @@
 maman|Derrière la boîte.
 narrateur|Le drap blanc reste contre la jambe, sage.
 papa|On a chuchoté ensemble.
-maman|La suite a eu sa place.</t>
+maman|On l'entend, maintenant.</t>
         </is>
       </c>
       <c r="AX20" t="inlineStr">
@@ -4777,17 +4777,17 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Dans le chuchotement, le mot a parlé. J'ai écouté, tout contre. Tes oreilles étaient à la bonne place. Le mur t'attend. Le drap blanc tient le carton, droit. Victorina essuie une main sur son pantalon. Une ombre reste sur le bois. Le loup avance, pas après pas.</t>
+          <t>Dans le chuchotement, le mot a parlé. J'ai écouté, tout contre. Tes oreilles étaient à la bonne place. Le mur t'attend. Le drap blanc tient le carton, droit. Victorina essuie une main sur son pantalon. Une ombre de drap reste sur le bois. Les oreilles du loup touchent le bois, sans bruit.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Dans le chuchotement, le mot a parlé. J'ai écouté, tout contre. Tes oreilles étaient à la bonne place. Le mur t'attend. Le drap blanc tient le carton, droit. Victorina essuie une main sur son pantalon. Une ombre reste sur le bois. Le &lt;emphasis level="moderate"&gt;loup&lt;/emphasis&gt; avance, pas après pas.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Dans le chuchotement, le mot a parlé. J'ai écouté, tout contre. Tes oreilles étaient à la bonne place. Le mur t'attend. Le drap blanc tient le carton, droit. Victorina essuie une main sur son pantalon. Une ombre de drap reste sur le bois. Les oreilles du &lt;emphasis level="moderate"&gt;loup&lt;/emphasis&gt; touchent le bois, sans bruit.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Dans le chuchotement, le mot a parlé. J'ai écouté, tout contre. Tes oreilles étaient à la bonne place. Le mur t'attend. Le drap blanc tient le carton, droit. Victorina essuie une main sur son pantalon. Une ombre reste sur le bois. Le &lt;emphasis&gt;loup&lt;/emphasis&gt; avance, pas après pas.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Dans le chuchotement, le mot a parlé. J'ai écouté, tout contre. Tes oreilles étaient à la bonne place. Le mur t'attend. Le drap blanc tient le carton, droit. Victorina essuie une main sur son pantalon. Une ombre de drap reste sur le bois. Les oreilles du &lt;emphasis&gt;loup&lt;/emphasis&gt; touchent le bois, sans bruit.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr"/>
@@ -4931,8 +4931,8 @@
 maman|Le mur t'attend.
 narrateur|Le drap blanc tient le carton, droit.
 narrateur|Victorina essuie une main sur son pantalon.
-narrateur|Une ombre reste sur le bois.
-narrateur|Le loup avance, pas après pas.</t>
+narrateur|Une ombre de drap reste sur le bois.
+narrateur|Les oreilles du loup touchent le bois, sans bruit.</t>
         </is>
       </c>
       <c r="AX21" t="inlineStr">
@@ -5148,17 +5148,17 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Sur la marche, la lune penche. Je l'ai vue, contre le fond. Le bois a gardé l'ombre. Rentre le carton, après le pas. Le drap blanc tient le carton, droit. Victorina souffle un peu sur les oreilles. Une poussière s'envole, puis retombe. La marche garde son ombre, seule.</t>
+          <t>Sur la marche, la lune penche. Je l'ai vue, contre le fond. Le bois a gardé l'ombre. Rentre le carton, après le pas. Le drap blanc tient le carton, droit. Victorina souffle un peu sur les oreilles. Une poussière s'envole, puis retombe. La marche garde une ombre de drap, seule.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Sur la marche, la lune penche. Je l'ai vue, contre le fond. Le bois a gardé l'ombre. Rentre le carton, après le pas. Le drap blanc tient le carton, droit. Victorina souffle un peu sur les oreilles. Une poussière s'envole, puis retombe. La marche garde son ombre, seule.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Sur la marche, la lune penche. Je l'ai vue, contre le fond. Le bois a gardé l'ombre. Rentre le carton, après le pas. Le drap blanc tient le carton, droit. Victorina souffle un peu sur les oreilles. Une poussière s'envole, puis retombe. La marche garde une ombre de drap, seule.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Sur la marche, la lune penche. Je l'ai vue, contre le fond. Le bois a gardé l'ombre. Rentre le carton, après le pas. Le drap blanc tient le carton, droit. Victorina souffle un peu sur les oreilles. Une poussière s'envole, puis retombe. La marche garde son ombre, seule.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Sur la marche, la lune penche. Je l'ai vue, contre le fond. Le bois a gardé l'ombre. Rentre le carton, après le pas. Le drap blanc tient le carton, droit. Victorina souffle un peu sur les oreilles. Une poussière s'envole, puis retombe. La marche garde une ombre de drap, seule.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr"/>
@@ -5303,7 +5303,7 @@
 narrateur|Le drap blanc tient le carton, droit.
 narrateur|Victorina souffle un peu sur les oreilles.
 narrateur|Une poussière s'envole, puis retombe.
-narrateur|La marche garde son ombre, seule.</t>
+narrateur|La marche garde une ombre de drap, seule.</t>
         </is>
       </c>
       <c r="AX23" t="inlineStr">
@@ -5904,17 +5904,17 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Sur le tabouret, Victorina a vu le cadre. Le mot est monté avec moi. Je remporte le tabouret, tout à l'heure. Essuie tes chaussettes, Victorina. Le drap blanc tient le carton, droit. Le loup marche jusqu'au palier. Une marche se tait, puis l'autre. L'étagère redevient calme, une planche.</t>
+          <t>Sur le tabouret, Victorina a vu le cadre. Le mot est monté avec moi. Je remporte le tabouret, tout à l'heure. Essuie tes chaussettes, Victorina. Le drap blanc tient le carton, droit. Le loup marche jusqu'au palier. Une marche se tait, puis l'autre. La planche du palier redevient une planche.</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Sur le tabouret, Victorina a vu le cadre. Le mot est monté avec moi. Je remporte le tabouret, tout à l'heure. Essuie tes chaussettes, Victorina. Le drap blanc tient le carton, droit. Le &lt;emphasis level="moderate"&gt;loup&lt;/emphasis&gt; marche jusqu'au palier. Une marche se tait, puis l'autre. L'étagère redevient calme, une planche.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Sur le tabouret, Victorina a vu le cadre. Le mot est monté avec moi. Je remporte le tabouret, tout à l'heure. Essuie tes chaussettes, Victorina. Le drap blanc tient le carton, droit. Le &lt;emphasis level="moderate"&gt;loup&lt;/emphasis&gt; marche jusqu'au palier. Une marche se tait, puis l'autre. La planche du palier redevient une planche.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Sur le tabouret, Victorina a vu le cadre. Le mot est monté avec moi. Je remporte le tabouret, tout à l'heure. Essuie tes chaussettes, Victorina. Le drap blanc tient le carton, droit. Le &lt;emphasis&gt;loup&lt;/emphasis&gt; marche jusqu'au palier. Une marche se tait, puis l'autre. L'étagère redevient calme, une planche.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Sur le tabouret, Victorina a vu le cadre. Le mot est monté avec moi. Je remporte le tabouret, tout à l'heure. Essuie tes chaussettes, Victorina. Le drap blanc tient le carton, droit. Le &lt;emphasis&gt;loup&lt;/emphasis&gt; marche jusqu'au palier. Une marche se tait, puis l'autre. La planche du palier redevient une planche.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr"/>
@@ -6059,7 +6059,7 @@
 narrateur|Le drap blanc tient le carton, droit.
 narrateur|Le loup marche jusqu'au palier.
 narrateur|Une marche se tait, puis l'autre.
-narrateur|L'étagère redevient calme, une planche.</t>
+narrateur|La planche du palier redevient une planche.</t>
         </is>
       </c>
       <c r="AX27" t="inlineStr">
@@ -6091,17 +6091,17 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Je regarde en bas. Victorina baisse les yeux, vers la plinthe. Pas le grand. Le petit, contre le bois. Une lune de papier penche, bas, tombée. Elle attendait près de la plinthe, sans un bruit. Le drap blanc reste contre la jambe, sage. Le mot a fini sa route. Merci d'avoir regardé jusque-là.</t>
+          <t>Je regarde en bas. Victorina baisse les yeux, vers la plinthe. Pas le grand. Le petit, contre le bois. Une lune de papier penche, bas, tombée. Elle attendait près de la plinthe, sans un bruit. Le drap blanc reste contre la jambe, sage. Elle attendait là, tout bas. Merci d'avoir baissé les yeux.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Je regarde en bas. Victorina baisse les yeux, vers la &lt;emphasis level="moderate"&gt;plinthe&lt;/emphasis&gt;. Pas le grand. Le petit, contre le bois. Une lune de papier penche, bas, tombée. Elle attendait près de la plinthe, sans un bruit. Le drap blanc reste contre la jambe, sage. Le mot a fini sa route. Merci d'avoir regardé jusque-là.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Je regarde en bas. Victorina baisse les yeux, vers la &lt;emphasis level="moderate"&gt;plinthe&lt;/emphasis&gt;. Pas le grand. Le petit, contre le bois. Une lune de papier penche, bas, tombée. Elle attendait près de la plinthe, sans un bruit. Le drap blanc reste contre la jambe, sage. Elle attendait là, tout bas. Merci d'avoir baissé les yeux.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Je regarde en bas. Victorina baisse les yeux, vers la &lt;emphasis&gt;plinthe&lt;/emphasis&gt;. Pas le grand. Le petit, contre le bois. Une lune de papier penche, bas, tombée. Elle attendait près de la plinthe, sans un bruit. Le drap blanc reste contre la jambe, sage. Le mot a fini sa route. Merci d'avoir regardé jusque-là. [pause]</t>
+          <t>Je regarde en bas. Victorina baisse les yeux, vers la &lt;emphasis&gt;plinthe&lt;/emphasis&gt;. Pas le grand. Le petit, contre le bois. Une lune de papier penche, bas, tombée. Elle attendait près de la plinthe, sans un bruit. Le drap blanc reste contre la jambe, sage. Elle attendait là, tout bas. Merci d'avoir baissé les yeux. [pause]</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr"/>
@@ -6242,8 +6242,8 @@
 narrateur|Une lune de papier penche, bas, tombée.
 narrateur|Elle attendait près de la plinthe, sans un bruit.
 narrateur|Le drap blanc reste contre la jambe, sage.
-maman|Le mot a fini sa route.
-papa|Merci d'avoir regardé jusque-là.</t>
+maman|Elle attendait là, tout bas.
+papa|Merci d'avoir baissé les yeux.</t>
         </is>
       </c>
       <c r="AX28" t="inlineStr">
@@ -6275,17 +6275,17 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Tout en bas, la lune brille, près de la plinthe. Tu as dit petit, à la fin. Merci d'avoir écouté jusque-là. Un peu de lait, après le mur. Le drap blanc tient le carton, droit. Victorina pose le carton contre le mur du palier. L'étagère reprend sa place, sage. Le haut n'a plus de secret, ce soir.</t>
+          <t>Tout en bas, la lune brille, près de la plinthe. Tu as dit petit, à la fin. Merci d'avoir regardé en bas. Le savon t'attend, près de l'eau. Le drap blanc tient le carton, droit. Victorina pose le carton contre le mur du palier. L'étagère reprend sa place, sage. Les carreaux du palier reprennent la bande jaune.</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Tout en bas, la lune brille, près de la plinthe. Tu as dit petit, à la fin. Merci d'avoir écouté jusque-là. Un peu de lait, après le mur. Le drap blanc tient le carton, droit. Victorina pose le carton contre le mur du palier. L'étagère reprend sa place, sage. Le haut n'a plus de secret, ce soir.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Tout en bas, la lune brille, près de la plinthe. Tu as dit petit, à la fin. Merci d'avoir regardé en bas. Le savon t'attend, près de l'eau. Le drap blanc tient le carton, droit. Victorina pose le carton contre le mur du palier. L'étagère reprend sa place, sage. Les carreaux du palier reprennent la bande jaune.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Tout en bas, la lune brille, près de la plinthe. Tu as dit petit, à la fin. Merci d'avoir écouté jusque-là. Un peu de lait, après le mur. Le drap blanc tient le carton, droit. Victorina pose le carton contre le mur du palier. L'étagère reprend sa place, sage. Le haut n'a plus de secret, ce soir.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Tout en bas, la lune brille, près de la plinthe. Tu as dit petit, à la fin. Merci d'avoir regardé en bas. Le savon t'attend, près de l'eau. Le drap blanc tient le carton, droit. Victorina pose le carton contre le mur du palier. L'étagère reprend sa place, sage. Les carreaux du palier reprennent la bande jaune.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr"/>
@@ -6425,12 +6425,12 @@
         <is>
           <t>narrateur|Tout en bas, la lune brille, près de la plinthe.
 enfant-f|Tu as dit petit, à la fin.
-papa|Merci d'avoir écouté jusque-là.
-maman|Un peu de lait, après le mur.
+papa|Merci d'avoir regardé en bas.
+maman|Le savon t'attend, près de l'eau.
 narrateur|Le drap blanc tient le carton, droit.
 narrateur|Victorina pose le carton contre le mur du palier.
 narrateur|L'étagère reprend sa place, sage.
-narrateur|Le haut n'a plus de secret, ce soir.</t>
+narrateur|Les carreaux du palier reprennent la bande jaune.</t>
         </is>
       </c>
       <c r="AX29" t="inlineStr">
@@ -6462,17 +6462,17 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Tes bras, papa. Viens, tout contre moi. Victorina s'élève, le nez au cadre, près des livres. La lune, tout près du bord. Je la vois ! Un rond blanc brille entre deux livres, enfin. Le drap blanc reste contre la jambe, sage. Tes bras ont fini la phrase. Chacun a fait sa part.</t>
+          <t>Tes bras, papa. Viens, tout contre moi. Victorina s'élève, le nez au cadre, près des livres. La lune, tout près du bord. Je la vois ! Un rond blanc brille entre deux livres, enfin. Le drap blanc reste contre la jambe, sage. Elle est entre les livres. Chacun a fait sa part.</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Tes &lt;emphasis level="moderate"&gt;bras&lt;/emphasis&gt;, papa. Viens, tout contre moi. Victorina s'élève, le nez au cadre, près des livres. La lune, tout près du bord. Je la vois ! Un rond blanc brille entre deux livres, enfin. Le drap blanc reste contre la jambe, sage. Tes bras ont fini la phrase. Chacun a fait sa part.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Tes &lt;emphasis level="moderate"&gt;bras&lt;/emphasis&gt;, papa. Viens, tout contre moi. Victorina s'élève, le nez au cadre, près des livres. La lune, tout près du bord. Je la vois ! Un rond blanc brille entre deux livres, enfin. Le drap blanc reste contre la jambe, sage. Elle est entre les livres. Chacun a fait sa part.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Tes &lt;emphasis&gt;bras&lt;/emphasis&gt;, papa. Viens, tout contre moi. Victorina s'élève, le nez au cadre, près des livres. La lune, tout près du bord. Je la vois ! Un rond blanc brille entre deux livres, enfin. Le drap blanc reste contre la jambe, sage. Tes bras ont fini la phrase. Chacun a fait sa part. [pause]</t>
+          <t>Tes &lt;emphasis&gt;bras&lt;/emphasis&gt;, papa. Viens, tout contre moi. Victorina s'élève, le nez au cadre, près des livres. La lune, tout près du bord. Je la vois ! Un rond blanc brille entre deux livres, enfin. Le drap blanc reste contre la jambe, sage. Elle est entre les livres. Chacun a fait sa part. [pause]</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr"/>
@@ -6613,7 +6613,7 @@
 enfant-f|Je la vois !
 narrateur|Un rond blanc brille entre deux livres, enfin.
 narrateur|Le drap blanc reste contre la jambe, sage.
-maman|Tes bras ont fini la phrase.
+maman|Elle est entre les livres.
 papa|Chacun a fait sa part.</t>
         </is>
       </c>
@@ -6646,17 +6646,17 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Dans les bras de papa, la lune était là. On l'a prise, tout haut. Tes yeux allaient assez loin. Le haut gardera son ombre. Le drap blanc tient le carton, droit. Victorina pose le carton près des carreaux. Les oreilles touchent l'air. Une bande jaune s'allonge, puis la lampe se tait.</t>
+          <t>Dans les bras de papa, la lune était là. On l'a prise, tout haut. Tes yeux allaient assez loin. Le haut gardera son ombre. Le drap blanc tient le carton, droit. Victorina pose le carton près des carreaux. Les oreilles touchent l'air. La bande jaune s'allonge, puis la lampe se tait.</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Dans les bras de papa, la lune était là. On l'a prise, tout haut. Tes yeux allaient assez loin. Le haut gardera son ombre. Le drap blanc tient le carton, droit. Victorina pose le carton près des carreaux. Les oreilles touchent l'air. Une bande jaune s'allonge, puis la lampe se tait.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Dans les bras de papa, la lune était là. On l'a prise, tout haut. Tes yeux allaient assez loin. Le haut gardera son ombre. Le drap blanc tient le carton, droit. Victorina pose le carton près des carreaux. Les oreilles touchent l'air. La bande jaune s'allonge, puis la lampe se tait.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Dans les bras de papa, la lune était là. On l'a prise, tout haut. Tes yeux allaient assez loin. Le haut gardera son ombre. Le drap blanc tient le carton, droit. Victorina pose le carton près des carreaux. Les oreilles touchent l'air. Une bande jaune s'allonge, puis la lampe se tait.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Dans les bras de papa, la lune était là. On l'a prise, tout haut. Tes yeux allaient assez loin. Le haut gardera son ombre. Le drap blanc tient le carton, droit. Victorina pose le carton près des carreaux. Les oreilles touchent l'air. La bande jaune s'allonge, puis la lampe se tait.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr"/>
@@ -6801,7 +6801,7 @@
 narrateur|Le drap blanc tient le carton, droit.
 narrateur|Victorina pose le carton près des carreaux.
 narrateur|Les oreilles touchent l'air.
-narrateur|Une bande jaune s'allonge, puis la lampe se tait.</t>
+narrateur|La bande jaune s'allonge, puis la lampe se tait.</t>
         </is>
       </c>
       <c r="AX31" t="inlineStr">
@@ -8154,17 +8154,17 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>La lune rentre derrière une oreille, un petit clic. Il marche, lui ! Sur le mur du buffet, les oreilles hautes. Bravo. Le loup de carton serre le bois. Une anse d'assiette garde un fil de colle. Le buffet redevient calme, autour des assiettes. Le savon de la cuisine sent, tiède.</t>
+          <t>La lune rentre derrière une oreille, un petit clic. Il marche, lui ! Sur le mur du buffet, les oreilles hautes. Regarde, il ne glisse plus. Le loup de carton serre le bois. Une anse d'assiette garde un fil de colle. Le buffet se tait autour des assiettes. Un fil de colle sèche sur une anse.</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La lune rentre derrière une oreille, un petit clic. Il marche, lui ! Sur le mur du buffet, les oreilles hautes. Bravo. Le &lt;emphasis level="moderate"&gt;loup&lt;/emphasis&gt; de carton serre le bois. Une anse d'assiette garde un fil de colle. Le buffet redevient calme, autour des assiettes. Le savon de la cuisine sent, tiède.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La lune rentre derrière une oreille, un petit clic. Il marche, lui ! Sur le mur du buffet, les oreilles hautes. Regarde, il ne glisse plus. Le &lt;emphasis level="moderate"&gt;loup&lt;/emphasis&gt; de carton serre le bois. Une anse d'assiette garde un fil de colle. Le buffet se tait autour des assiettes. Un fil de colle sèche sur une anse.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La lune rentre derrière une oreille, un petit clic. Il marche, lui ! Sur le mur du buffet, les oreilles hautes. Bravo. Le &lt;emphasis&gt;loup&lt;/emphasis&gt; de carton serre le bois. Une anse d'assiette garde un fil de colle. Le buffet redevient calme, autour des assiettes. Le savon de la cuisine sent, tiède.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La lune rentre derrière une oreille, un petit clic. Il marche, lui ! Sur le mur du buffet, les oreilles hautes. Regarde, il ne glisse plus. Le &lt;emphasis&gt;loup&lt;/emphasis&gt; de carton serre le bois. Une anse d'assiette garde un fil de colle. Le buffet se tait autour des assiettes. Un fil de colle sèche sur une anse.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr"/>
@@ -8305,11 +8305,11 @@
           <t>narrateur|La lune rentre derrière une oreille, un petit clic.
 enfant-f|Il marche, lui !
 papa|Sur le mur du buffet, les oreilles hautes.
-maman|Bravo.
+maman|Regarde, il ne glisse plus.
 narrateur|Le loup de carton serre le bois.
 narrateur|Une anse d'assiette garde un fil de colle.
-narrateur|Le buffet redevient calme, autour des assiettes.
-narrateur|Le savon de la cuisine sent, tiède.</t>
+narrateur|Le buffet se tait autour des assiettes.
+narrateur|Un fil de colle sèche sur une anse.</t>
         </is>
       </c>
       <c r="AX39" t="inlineStr">
@@ -8525,17 +8525,17 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Le loup part entre deux ombres d'assiettes. J'ai posé la serviette, lui d'abord. Puis le mot est venu. Venez, le mur est prêt. Le loup de carton serre le bois. Victorina redresse une oreille, du pouce. Une assiette tinte, puis se tait. Le couloir laisse un rai, mince.</t>
+          <t>Le loup part entre deux ombres d'assiettes. J'ai posé la serviette, lui d'abord. Puis le mot est venu. Venez, le mur est prêt. Le loup de carton serre le bois. Victorina redresse une oreille, du pouce. Une assiette tinte, puis se tait. Le couloir laisse un rai sur le carton gris.</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le &lt;emphasis level="moderate"&gt;loup&lt;/emphasis&gt; part entre deux ombres d'assiettes. J'ai posé la serviette, lui d'abord. Puis le mot est venu. Venez, le mur est prêt. Le loup de carton serre le bois. Victorina redresse une oreille, du pouce. Une assiette tinte, puis se tait. Le couloir laisse un rai, mince.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le &lt;emphasis level="moderate"&gt;loup&lt;/emphasis&gt; part entre deux ombres d'assiettes. J'ai posé la serviette, lui d'abord. Puis le mot est venu. Venez, le mur est prêt. Le loup de carton serre le bois. Victorina redresse une oreille, du pouce. Une assiette tinte, puis se tait. Le couloir laisse un rai sur le carton gris.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le &lt;emphasis&gt;loup&lt;/emphasis&gt; part entre deux ombres d'assiettes. J'ai posé la serviette, lui d'abord. Puis le mot est venu. Venez, le mur est prêt. Le loup de carton serre le bois. Victorina redresse une oreille, du pouce. Une assiette tinte, puis se tait. Le couloir laisse un rai, mince.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le &lt;emphasis&gt;loup&lt;/emphasis&gt; part entre deux ombres d'assiettes. J'ai posé la serviette, lui d'abord. Puis le mot est venu. Venez, le mur est prêt. Le loup de carton serre le bois. Victorina redresse une oreille, du pouce. Une assiette tinte, puis se tait. Le couloir laisse un rai sur le carton gris.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr"/>
@@ -8680,7 +8680,7 @@
 narrateur|Le loup de carton serre le bois.
 narrateur|Victorina redresse une oreille, du pouce.
 narrateur|Une assiette tinte, puis se tait.
-narrateur|Le couloir laisse un rai, mince.</t>
+narrateur|Le couloir laisse un rai sur le carton gris.</t>
         </is>
       </c>
       <c r="AX41" t="inlineStr">
@@ -8896,17 +8896,17 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Contre la chaise, le loup tient, museau bas. On s'est assis, lui sur moi. Le haut gardera son ombre. Tiens bien le carton. Le loup de carton serre le bois. Victorina gratte un peu de colle, du doigt. Une poussière s'envole, puis retombe. Une horloge tape, puis le buffet se tait.</t>
+          <t>Contre la chaise, le loup tient, museau bas. On s'est assis, lui sur moi. Le haut gardera son ombre. Tiens bien le carton. Le loup de carton serre le bois. Victorina gratte un peu de colle, du doigt. Une poussière s'envole, puis retombe. L'horloge tape, et le museau se tient.</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Contre la chaise, le &lt;emphasis level="moderate"&gt;loup&lt;/emphasis&gt; tient, museau bas. On s'est assis, lui sur moi. Le haut gardera son ombre. Tiens bien le carton. Le loup de carton serre le bois. Victorina gratte un peu de colle, du doigt. Une poussière s'envole, puis retombe. Une horloge tape, puis le buffet se tait.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Contre la chaise, le &lt;emphasis level="moderate"&gt;loup&lt;/emphasis&gt; tient, museau bas. On s'est assis, lui sur moi. Le haut gardera son ombre. Tiens bien le carton. Le loup de carton serre le bois. Victorina gratte un peu de colle, du doigt. Une poussière s'envole, puis retombe. L'horloge tape, et le museau se tient.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Contre la chaise, le &lt;emphasis&gt;loup&lt;/emphasis&gt; tient, museau bas. On s'est assis, lui sur moi. Le haut gardera son ombre. Tiens bien le carton. Le loup de carton serre le bois. Victorina gratte un peu de colle, du doigt. Une poussière s'envole, puis retombe. Une horloge tape, puis le buffet se tait.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Contre la chaise, le &lt;emphasis&gt;loup&lt;/emphasis&gt; tient, museau bas. On s'est assis, lui sur moi. Le haut gardera son ombre. Tiens bien le carton. Le loup de carton serre le bois. Victorina gratte un peu de colle, du doigt. Une poussière s'envole, puis retombe. L'horloge tape, et le museau se tient.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr"/>
@@ -9051,7 +9051,7 @@
 narrateur|Le loup de carton serre le bois.
 narrateur|Victorina gratte un peu de colle, du doigt.
 narrateur|Une poussière s'envole, puis retombe.
-narrateur|Une horloge tape, puis le buffet se tait.</t>
+narrateur|L'horloge tape, et le museau se tient.</t>
         </is>
       </c>
       <c r="AX43" t="inlineStr">
@@ -9652,17 +9652,17 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Loin de l'écho, la lune était collée au carton. Tu as fini, papa. Oui, le mot était long. Tu as tenu la porte. Le loup de carton serre le bois. Une poussière sèche sur une oreille. Victorina fait marcher le loup, près du bois. Le placard redevient un placard, simple.</t>
+          <t>Loin de l'écho, la lune était collée au carton. Tu as fini, papa. Oui, le mot était long. Tu as tenu la porte. Le loup de carton serre le bois. Une poussière sèche sur une oreille. Victorina fait marcher le loup, près du bois. Le placard referme son écho, sans un mot.</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Loin de l'écho, la lune était collée au carton. Tu as fini, papa. Oui, le mot était long. Tu as tenu la porte. Le &lt;emphasis level="moderate"&gt;loup&lt;/emphasis&gt; de carton serre le bois. Une poussière sèche sur une oreille. Victorina fait marcher le loup, près du bois. Le placard redevient un placard, simple.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Loin de l'écho, la lune était collée au carton. Tu as fini, papa. Oui, le mot était long. Tu as tenu la porte. Le &lt;emphasis level="moderate"&gt;loup&lt;/emphasis&gt; de carton serre le bois. Une poussière sèche sur une oreille. Victorina fait marcher le loup, près du bois. Le placard referme son écho, sans un mot.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Loin de l'écho, la lune était collée au carton. Tu as fini, papa. Oui, le mot était long. Tu as tenu la porte. Le &lt;emphasis&gt;loup&lt;/emphasis&gt; de carton serre le bois. Une poussière sèche sur une oreille. Victorina fait marcher le loup, près du bois. Le placard redevient un placard, simple.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Loin de l'écho, la lune était collée au carton. Tu as fini, papa. Oui, le mot était long. Tu as tenu la porte. Le &lt;emphasis&gt;loup&lt;/emphasis&gt; de carton serre le bois. Une poussière sèche sur une oreille. Victorina fait marcher le loup, près du bois. Le placard referme son écho, sans un mot.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr"/>
@@ -9807,7 +9807,7 @@
 narrateur|Le loup de carton serre le bois.
 narrateur|Une poussière sèche sur une oreille.
 narrateur|Victorina fait marcher le loup, près du bois.
-narrateur|Le placard redevient un placard, simple.</t>
+narrateur|Le placard referme son écho, sans un mot.</t>
         </is>
       </c>
       <c r="AX47" t="inlineStr">
@@ -9839,17 +9839,17 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Chut, loup. Tout près des oreilles. L'écho recule, et le carton ne gratte plus. Derrière. Victorina colle le loup à sa joue, silencieuse. Derrière la boîte. Le loup de carton attend un dernier pas. On a chuchoté ensemble. La suite a eu sa place.</t>
+          <t>Chut, loup. Tout près des oreilles. L'écho recule, et le carton ne gratte plus. Derrière. Victorina colle le loup à sa joue, silencieuse. Derrière la boîte. Le loup de carton attend un dernier pas. On a chuchoté ensemble. On l'entend, maintenant.</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Chut, loup. Tout près des oreilles. L'écho recule, et le carton ne gratte plus. Derrière. Victorina colle le loup à sa joue, silencieuse. Derrière la boîte. Le loup de carton attend un dernier pas. On a chuchoté ensemble. La suite a eu sa place.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Chut, loup. Tout près des oreilles. L'écho recule, et le carton ne gratte plus. Derrière. Victorina colle le loup à sa joue, silencieuse. Derrière la boîte. Le loup de carton attend un dernier pas. On a chuchoté ensemble. On l'entend, maintenant.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Chut, loup. Tout près des oreilles. L'écho recule, et le carton ne gratte plus. Derrière. Victorina colle le loup à sa joue, silencieuse. Derrière la boîte. Le loup de carton attend un dernier pas. On a chuchoté ensemble. La suite a eu sa place. [pause]</t>
+          <t>Chut, loup. Tout près des oreilles. L'écho recule, et le carton ne gratte plus. Derrière. Victorina colle le loup à sa joue, silencieuse. Derrière la boîte. Le loup de carton attend un dernier pas. On a chuchoté ensemble. On l'entend, maintenant. [pause]</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr"/>
@@ -9991,7 +9991,7 @@
 maman|Derrière la boîte.
 narrateur|Le loup de carton attend un dernier pas.
 papa|On a chuchoté ensemble.
-maman|La suite a eu sa place.</t>
+maman|On l'entend, maintenant.</t>
         </is>
       </c>
       <c r="AX48" t="inlineStr">
@@ -10023,17 +10023,17 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Dans le chuchotement, le loup a entendu la fin. J'ai collé mon oreille, tout contre. Tes oreilles étaient à la bonne place. Le mur t'attend. Le loup de carton serre le bois. Victorina essuie la colle sur son pantalon. Une ombre d'oreille reste sur le bois. Le loup avance, pas après pas.</t>
+          <t>Dans le chuchotement, le loup a entendu la fin. J'ai collé mon oreille, tout contre. Tes oreilles étaient à la bonne place. Le mur t'attend. Le loup de carton serre le bois. Victorina essuie la colle sur son pantalon. Une ombre d'oreille reste sur le bois. Le loup avance, oreilles hautes, pas après pas.</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Dans le chuchotement, le &lt;emphasis level="moderate"&gt;loup&lt;/emphasis&gt; a entendu la fin. J'ai collé mon oreille, tout contre. Tes oreilles étaient à la bonne place. Le mur t'attend. Le loup de carton serre le bois. Victorina essuie la colle sur son pantalon. Une ombre d'oreille reste sur le bois. Le loup avance, pas après pas.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Dans le chuchotement, le &lt;emphasis level="moderate"&gt;loup&lt;/emphasis&gt; a entendu la fin. J'ai collé mon oreille, tout contre. Tes oreilles étaient à la bonne place. Le mur t'attend. Le loup de carton serre le bois. Victorina essuie la colle sur son pantalon. Une ombre d'oreille reste sur le bois. Le loup avance, oreilles hautes, pas après pas.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Dans le chuchotement, le &lt;emphasis&gt;loup&lt;/emphasis&gt; a entendu la fin. J'ai collé mon oreille, tout contre. Tes oreilles étaient à la bonne place. Le mur t'attend. Le loup de carton serre le bois. Victorina essuie la colle sur son pantalon. Une ombre d'oreille reste sur le bois. Le loup avance, pas après pas.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Dans le chuchotement, le &lt;emphasis&gt;loup&lt;/emphasis&gt; a entendu la fin. J'ai collé mon oreille, tout contre. Tes oreilles étaient à la bonne place. Le mur t'attend. Le loup de carton serre le bois. Victorina essuie la colle sur son pantalon. Une ombre d'oreille reste sur le bois. Le loup avance, oreilles hautes, pas après pas.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr"/>
@@ -10178,7 +10178,7 @@
 narrateur|Le loup de carton serre le bois.
 narrateur|Victorina essuie la colle sur son pantalon.
 narrateur|Une ombre d'oreille reste sur le bois.
-narrateur|Le loup avance, pas après pas.</t>
+narrateur|Le loup avance, oreilles hautes, pas après pas.</t>
         </is>
       </c>
       <c r="AX49" t="inlineStr">
@@ -10394,17 +10394,17 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Sur la marche, la lune penche vers le museau. Il l'a vue, contre le fond. Le bois a gardé l'ombre. Rentre le carton, après le pas. Le loup de carton serre le bois. Victorina souffle un peu sur les oreilles. Une poussière s'envole, puis retombe. La marche garde son ombre, seule.</t>
+          <t>Sur la marche, la lune penche vers le museau. Il l'a vue, contre le fond. Le bois a gardé l'ombre. Rentre le carton, après le pas. Le loup de carton serre le bois. Victorina souffle un peu sur les oreilles. Une poussière s'envole, puis retombe. La marche garde une ombre de museau, seule.</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Sur la marche, la lune penche vers le museau. Il l'a vue, contre le fond. Le bois a gardé l'ombre. Rentre le carton, après le pas. Le &lt;emphasis level="moderate"&gt;loup&lt;/emphasis&gt; de carton serre le bois. Victorina souffle un peu sur les oreilles. Une poussière s'envole, puis retombe. La marche garde son ombre, seule.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Sur la marche, la lune penche vers le museau. Il l'a vue, contre le fond. Le bois a gardé l'ombre. Rentre le carton, après le pas. Le &lt;emphasis level="moderate"&gt;loup&lt;/emphasis&gt; de carton serre le bois. Victorina souffle un peu sur les oreilles. Une poussière s'envole, puis retombe. La marche garde une ombre de museau, seule.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Sur la marche, la lune penche vers le museau. Il l'a vue, contre le fond. Le bois a gardé l'ombre. Rentre le carton, après le pas. Le &lt;emphasis&gt;loup&lt;/emphasis&gt; de carton serre le bois. Victorina souffle un peu sur les oreilles. Une poussière s'envole, puis retombe. La marche garde son ombre, seule.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Sur la marche, la lune penche vers le museau. Il l'a vue, contre le fond. Le bois a gardé l'ombre. Rentre le carton, après le pas. Le &lt;emphasis&gt;loup&lt;/emphasis&gt; de carton serre le bois. Victorina souffle un peu sur les oreilles. Une poussière s'envole, puis retombe. La marche garde une ombre de museau, seule.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr"/>
@@ -10549,7 +10549,7 @@
 narrateur|Le loup de carton serre le bois.
 narrateur|Victorina souffle un peu sur les oreilles.
 narrateur|Une poussière s'envole, puis retombe.
-narrateur|La marche garde son ombre, seule.</t>
+narrateur|La marche garde une ombre de museau, seule.</t>
         </is>
       </c>
       <c r="AX51" t="inlineStr">
@@ -11150,17 +11150,17 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>Sur le tabouret, le loup a vu le cadre. Le mot est monté avec nous. Je remporte le tabouret, tout à l'heure. Essuie tes chaussettes, Victorina. Le loup de carton serre le bois. Le loup marche jusqu'au palier, oreilles hautes. Une marche se tait, puis l'autre. L'étagère redevient calme, une planche.</t>
+          <t>Sur le tabouret, le loup a vu le cadre. Le mot est monté avec nous. Je remporte le tabouret, tout à l'heure. Essuie tes chaussettes, Victorina. Le loup de carton serre le bois. Le loup marche jusqu'au palier, oreilles hautes. Une marche se tait, puis l'autre. Deux oreilles passent la planche, puis s'arrêtent.</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Sur le tabouret, le &lt;emphasis level="moderate"&gt;loup&lt;/emphasis&gt; a vu le cadre. Le mot est monté avec nous. Je remporte le tabouret, tout à l'heure. Essuie tes chaussettes, Victorina. Le loup de carton serre le bois. Le loup marche jusqu'au palier, oreilles hautes. Une marche se tait, puis l'autre. L'étagère redevient calme, une planche.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Sur le tabouret, le &lt;emphasis level="moderate"&gt;loup&lt;/emphasis&gt; a vu le cadre. Le mot est monté avec nous. Je remporte le tabouret, tout à l'heure. Essuie tes chaussettes, Victorina. Le loup de carton serre le bois. Le loup marche jusqu'au palier, oreilles hautes. Une marche se tait, puis l'autre. Deux oreilles passent la planche, puis s'arrêtent.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Sur le tabouret, le &lt;emphasis&gt;loup&lt;/emphasis&gt; a vu le cadre. Le mot est monté avec nous. Je remporte le tabouret, tout à l'heure. Essuie tes chaussettes, Victorina. Le loup de carton serre le bois. Le loup marche jusqu'au palier, oreilles hautes. Une marche se tait, puis l'autre. L'étagère redevient calme, une planche.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Sur le tabouret, le &lt;emphasis&gt;loup&lt;/emphasis&gt; a vu le cadre. Le mot est monté avec nous. Je remporte le tabouret, tout à l'heure. Essuie tes chaussettes, Victorina. Le loup de carton serre le bois. Le loup marche jusqu'au palier, oreilles hautes. Une marche se tait, puis l'autre. Deux oreilles passent la planche, puis s'arrêtent.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr"/>
@@ -11305,7 +11305,7 @@
 narrateur|Le loup de carton serre le bois.
 narrateur|Le loup marche jusqu'au palier, oreilles hautes.
 narrateur|Une marche se tait, puis l'autre.
-narrateur|L'étagère redevient calme, une planche.</t>
+narrateur|Deux oreilles passent la planche, puis s'arrêtent.</t>
         </is>
       </c>
       <c r="AX55" t="inlineStr">
@@ -11337,17 +11337,17 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Le loup regarde en bas. Victorina baisse le carton, vers la plinthe. Pas le grand. Le petit, contre le bois. Une lune de papier penche, bas, tombée. Le museau la touche, sans la froisser. Le loup de carton attend un dernier pas. Le mot a fini sa route. Merci d'avoir regardé jusque-là.</t>
+          <t>Le loup regarde en bas. Victorina baisse le carton, vers la plinthe. Pas le grand. Le petit, contre le bois. Une lune de papier penche, bas, tombée. Le museau la touche, sans la froisser. Le loup de carton attend un dernier pas. Elle attendait là, tout bas. Merci d'avoir baissé les yeux.</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le loup regarde en bas. Victorina baisse le carton, vers la &lt;emphasis level="moderate"&gt;plinthe&lt;/emphasis&gt;. Pas le grand. Le petit, contre le bois. Une lune de papier penche, bas, tombée. Le museau la touche, sans la froisser. Le loup de carton attend un dernier pas. Le mot a fini sa route. Merci d'avoir regardé jusque-là.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le loup regarde en bas. Victorina baisse le carton, vers la &lt;emphasis level="moderate"&gt;plinthe&lt;/emphasis&gt;. Pas le grand. Le petit, contre le bois. Une lune de papier penche, bas, tombée. Le museau la touche, sans la froisser. Le loup de carton attend un dernier pas. Elle attendait là, tout bas. Merci d'avoir baissé les yeux.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Le loup regarde en bas. Victorina baisse le carton, vers la &lt;emphasis&gt;plinthe&lt;/emphasis&gt;. Pas le grand. Le petit, contre le bois. Une lune de papier penche, bas, tombée. Le museau la touche, sans la froisser. Le loup de carton attend un dernier pas. Le mot a fini sa route. Merci d'avoir regardé jusque-là. [pause]</t>
+          <t>Le loup regarde en bas. Victorina baisse le carton, vers la &lt;emphasis&gt;plinthe&lt;/emphasis&gt;. Pas le grand. Le petit, contre le bois. Une lune de papier penche, bas, tombée. Le museau la touche, sans la froisser. Le loup de carton attend un dernier pas. Elle attendait là, tout bas. Merci d'avoir baissé les yeux. [pause]</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr"/>
@@ -11488,8 +11488,8 @@
 narrateur|Une lune de papier penche, bas, tombée.
 narrateur|Le museau la touche, sans la froisser.
 narrateur|Le loup de carton attend un dernier pas.
-maman|Le mot a fini sa route.
-papa|Merci d'avoir regardé jusque-là.</t>
+maman|Elle attendait là, tout bas.
+papa|Merci d'avoir baissé les yeux.</t>
         </is>
       </c>
       <c r="AX56" t="inlineStr">
@@ -11521,17 +11521,17 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Tout en bas, la lune brille, près du museau. Tu as dit petit, à la fin. Merci d'avoir écouté jusque-là. Un peu de lait, après le mur. Le loup de carton serre le bois. Victorina pose le carton contre le mur du palier. L'étagère reprend sa place, sage. Le haut n'a plus de secret, ce soir.</t>
+          <t>Tout en bas, la lune brille, près du museau. Tu as dit petit, à la fin. Merci d'avoir regardé en bas. Le savon t'attend, près de l'eau. Le loup de carton serre le bois. Victorina pose le carton contre le mur du palier. L'étagère reprend sa place, sage. Le haut n'a plus rien à cacher, ce soir.</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Tout en bas, la lune brille, près du museau. Tu as dit petit, à la fin. Merci d'avoir écouté jusque-là. Un peu de lait, après le mur. Le &lt;emphasis level="moderate"&gt;loup&lt;/emphasis&gt; de carton serre le bois. Victorina pose le carton contre le mur du palier. L'étagère reprend sa place, sage. Le haut n'a plus de secret, ce soir.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Tout en bas, la lune brille, près du museau. Tu as dit petit, à la fin. Merci d'avoir regardé en bas. Le savon t'attend, près de l'eau. Le &lt;emphasis level="moderate"&gt;loup&lt;/emphasis&gt; de carton serre le bois. Victorina pose le carton contre le mur du palier. L'étagère reprend sa place, sage. Le haut n'a plus rien à cacher, ce soir.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Tout en bas, la lune brille, près du museau. Tu as dit petit, à la fin. Merci d'avoir écouté jusque-là. Un peu de lait, après le mur. Le &lt;emphasis&gt;loup&lt;/emphasis&gt; de carton serre le bois. Victorina pose le carton contre le mur du palier. L'étagère reprend sa place, sage. Le haut n'a plus de secret, ce soir.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Tout en bas, la lune brille, près du museau. Tu as dit petit, à la fin. Merci d'avoir regardé en bas. Le savon t'attend, près de l'eau. Le &lt;emphasis&gt;loup&lt;/emphasis&gt; de carton serre le bois. Victorina pose le carton contre le mur du palier. L'étagère reprend sa place, sage. Le haut n'a plus rien à cacher, ce soir.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr"/>
@@ -11671,12 +11671,12 @@
         <is>
           <t>narrateur|Tout en bas, la lune brille, près du museau.
 enfant-f|Tu as dit petit, à la fin.
-papa|Merci d'avoir écouté jusque-là.
-maman|Un peu de lait, après le mur.
+papa|Merci d'avoir regardé en bas.
+maman|Le savon t'attend, près de l'eau.
 narrateur|Le loup de carton serre le bois.
 narrateur|Victorina pose le carton contre le mur du palier.
 narrateur|L'étagère reprend sa place, sage.
-narrateur|Le haut n'a plus de secret, ce soir.</t>
+narrateur|Le haut n'a plus rien à cacher, ce soir.</t>
         </is>
       </c>
       <c r="AX57" t="inlineStr">
@@ -11708,17 +11708,17 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Tes bras, et le loup. Viens, tout contre moi. Victorina s'élève, le carton entre eux, près des livres. La lune, tout près du bord. Il la voit ! Un rond blanc brille entre deux livres, enfin. Le loup de carton attend un dernier pas. Tes bras ont fini la phrase. Chacun a fait sa part.</t>
+          <t>Tes bras, et le loup. Viens, tout contre moi. Victorina s'élève, le carton entre eux, près des livres. La lune, tout près du bord. Il la voit ! Un rond blanc brille entre deux livres, enfin. Le loup de carton attend un dernier pas. Elle est entre les livres. Chacun a fait sa part.</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Tes &lt;emphasis level="moderate"&gt;bras&lt;/emphasis&gt;, et le loup. Viens, tout contre moi. Victorina s'élève, le carton entre eux, près des livres. La lune, tout près du bord. Il la voit ! Un rond blanc brille entre deux livres, enfin. Le loup de carton attend un dernier pas. Tes bras ont fini la phrase. Chacun a fait sa part.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Tes &lt;emphasis level="moderate"&gt;bras&lt;/emphasis&gt;, et le loup. Viens, tout contre moi. Victorina s'élève, le carton entre eux, près des livres. La lune, tout près du bord. Il la voit ! Un rond blanc brille entre deux livres, enfin. Le loup de carton attend un dernier pas. Elle est entre les livres. Chacun a fait sa part.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Tes &lt;emphasis&gt;bras&lt;/emphasis&gt;, et le loup. Viens, tout contre moi. Victorina s'élève, le carton entre eux, près des livres. La lune, tout près du bord. Il la voit ! Un rond blanc brille entre deux livres, enfin. Le loup de carton attend un dernier pas. Tes bras ont fini la phrase. Chacun a fait sa part. [pause]</t>
+          <t>Tes &lt;emphasis&gt;bras&lt;/emphasis&gt;, et le loup. Viens, tout contre moi. Victorina s'élève, le carton entre eux, près des livres. La lune, tout près du bord. Il la voit ! Un rond blanc brille entre deux livres, enfin. Le loup de carton attend un dernier pas. Elle est entre les livres. Chacun a fait sa part. [pause]</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr"/>
@@ -11859,7 +11859,7 @@
 enfant-f|Il la voit !
 narrateur|Un rond blanc brille entre deux livres, enfin.
 narrateur|Le loup de carton attend un dernier pas.
-maman|Tes bras ont fini la phrase.
+maman|Elle est entre les livres.
 papa|Chacun a fait sa part.</t>
         </is>
       </c>
@@ -11892,17 +11892,17 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Dans les bras de papa, le loup a pris la lune. On l'a prise, tout haut. Tes yeux allaient assez loin. Le haut gardera son ombre. Le loup de carton serre le bois. Victorina pose le carton près des carreaux. Les oreilles touchent l'air. Une bande jaune s'allonge, puis la lampe se tait.</t>
+          <t>Dans les bras de papa, le loup a pris la lune. On l'a prise, tout haut. Tes yeux allaient assez loin. Le haut gardera son ombre. Le loup de carton serre le bois. Victorina pose le carton près des carreaux. Les oreilles touchent l'air, près des carreaux. La lampe du portemanteau tient un rond, puis s'éteint.</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Dans les bras de papa, le &lt;emphasis level="moderate"&gt;loup&lt;/emphasis&gt; a pris la lune. On l'a prise, tout haut. Tes yeux allaient assez loin. Le haut gardera son ombre. Le loup de carton serre le bois. Victorina pose le carton près des carreaux. Les oreilles touchent l'air. Une bande jaune s'allonge, puis la lampe se tait.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Dans les bras de papa, le &lt;emphasis level="moderate"&gt;loup&lt;/emphasis&gt; a pris la lune. On l'a prise, tout haut. Tes yeux allaient assez loin. Le haut gardera son ombre. Le loup de carton serre le bois. Victorina pose le carton près des carreaux. Les oreilles touchent l'air, près des carreaux. La lampe du portemanteau tient un rond, puis s'éteint.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Dans les bras de papa, le &lt;emphasis&gt;loup&lt;/emphasis&gt; a pris la lune. On l'a prise, tout haut. Tes yeux allaient assez loin. Le haut gardera son ombre. Le loup de carton serre le bois. Victorina pose le carton près des carreaux. Les oreilles touchent l'air. Une bande jaune s'allonge, puis la lampe se tait.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Dans les bras de papa, le &lt;emphasis&gt;loup&lt;/emphasis&gt; a pris la lune. On l'a prise, tout haut. Tes yeux allaient assez loin. Le haut gardera son ombre. Le loup de carton serre le bois. Victorina pose le carton près des carreaux. Les oreilles touchent l'air, près des carreaux. La lampe du portemanteau tient un rond, puis s'éteint.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr"/>
@@ -12046,8 +12046,8 @@
 maman|Le haut gardera son ombre.
 narrateur|Le loup de carton serre le bois.
 narrateur|Victorina pose le carton près des carreaux.
-narrateur|Les oreilles touchent l'air.
-narrateur|Une bande jaune s'allonge, puis la lampe se tait.</t>
+narrateur|Les oreilles touchent l'air, près des carreaux.
+narrateur|La lampe du portemanteau tient un rond, puis s'éteint.</t>
         </is>
       </c>
       <c r="AX59" t="inlineStr">
@@ -13399,17 +13399,17 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>La lune rentre dans le rond, un petit clic. Il marche, dans la lumière ! Sur le mur du buffet, le rond le suit. Bravo. La lampe ronde cliquette une fois, puis se tait. Une miette sèche dans le cercle jaune. Le buffet redevient calme, autour des assiettes. Le savon de la cuisine sent, tiède.</t>
+          <t>La lune rentre dans le rond, un petit clic. Il marche, dans la lumière ! Sur le mur du buffet, le rond le suit. Le rond le tient, maintenant. La lampe ronde cliquette une fois, puis se tait. Une miette sèche dans le cercle jaune. Le buffet se tait autour des assiettes. Le savon sent, et le rond s'éteint.</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La lune rentre dans le rond, un petit clic. Il marche, dans la lumière ! Sur le mur du buffet, le rond le suit. Bravo. La lampe ronde cliquette une fois, puis se tait. Une miette sèche dans le cercle jaune. Le buffet redevient calme, autour des assiettes. Le savon de la cuisine sent, tiède.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La lune rentre dans le rond, un petit clic. Il marche, dans la lumière ! Sur le mur du buffet, le rond le suit. Le rond le tient, maintenant. La lampe ronde cliquette une fois, puis se tait. Une miette sèche dans le cercle jaune. Le buffet se tait autour des assiettes. Le savon sent, et le rond s'éteint.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La lune rentre dans le rond, un petit clic. Il marche, dans la lumière ! Sur le mur du buffet, le rond le suit. Bravo. La lampe ronde cliquette une fois, puis se tait. Une miette sèche dans le cercle jaune. Le buffet redevient calme, autour des assiettes. Le savon de la cuisine sent, tiède.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La lune rentre dans le rond, un petit clic. Il marche, dans la lumière ! Sur le mur du buffet, le rond le suit. Le rond le tient, maintenant. La lampe ronde cliquette une fois, puis se tait. Une miette sèche dans le cercle jaune. Le buffet se tait autour des assiettes. Le savon sent, et le rond s'éteint.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr"/>
@@ -13550,11 +13550,11 @@
           <t>narrateur|La lune rentre dans le rond, un petit clic.
 enfant-f|Il marche, dans la lumière !
 papa|Sur le mur du buffet, le rond le suit.
-maman|Bravo.
+maman|Le rond le tient, maintenant.
 narrateur|La lampe ronde cliquette une fois, puis se tait.
 narrateur|Une miette sèche dans le cercle jaune.
-narrateur|Le buffet redevient calme, autour des assiettes.
-narrateur|Le savon de la cuisine sent, tiède.</t>
+narrateur|Le buffet se tait autour des assiettes.
+narrateur|Le savon sent, et le rond s'éteint.</t>
         </is>
       </c>
       <c r="AX67" t="inlineStr">
@@ -13770,17 +13770,17 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>Le loup part, gris, dans le rond des assiettes. J'ai posé la serviette, sans clic. Puis le mot est venu. Venez, le mur est prêt. La lampe ronde cliquette une fois, puis se tait. Victorina pose le carton contre l'épaule. Une assiette tinte, puis se tait. Le couloir laisse un rai, mince.</t>
+          <t>Le loup part, gris, dans le rond des assiettes. J'ai posé la serviette, sans clic. Puis le mot est venu. Venez, le mur est prêt. La lampe ronde cliquette une fois, puis se tait. Victorina pose le carton contre l'épaule. Une assiette tinte, puis se tait. Un rai mince dort dans le verre de la lampe.</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le &lt;emphasis level="moderate"&gt;loup&lt;/emphasis&gt; part, gris, dans le rond des assiettes. J'ai posé la serviette, sans clic. Puis le mot est venu. Venez, le mur est prêt. La lampe ronde cliquette une fois, puis se tait. Victorina pose le carton contre l'épaule. Une assiette tinte, puis se tait. Le couloir laisse un rai, mince.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le &lt;emphasis level="moderate"&gt;loup&lt;/emphasis&gt; part, gris, dans le rond des assiettes. J'ai posé la serviette, sans clic. Puis le mot est venu. Venez, le mur est prêt. La lampe ronde cliquette une fois, puis se tait. Victorina pose le carton contre l'épaule. Une assiette tinte, puis se tait. Un rai mince dort dans le verre de la lampe.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le &lt;emphasis&gt;loup&lt;/emphasis&gt; part, gris, dans le rond des assiettes. J'ai posé la serviette, sans clic. Puis le mot est venu. Venez, le mur est prêt. La lampe ronde cliquette une fois, puis se tait. Victorina pose le carton contre l'épaule. Une assiette tinte, puis se tait. Le couloir laisse un rai, mince.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le &lt;emphasis&gt;loup&lt;/emphasis&gt; part, gris, dans le rond des assiettes. J'ai posé la serviette, sans clic. Puis le mot est venu. Venez, le mur est prêt. La lampe ronde cliquette une fois, puis se tait. Victorina pose le carton contre l'épaule. Une assiette tinte, puis se tait. Un rai mince dort dans le verre de la lampe.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr"/>
@@ -13925,7 +13925,7 @@
 narrateur|La lampe ronde cliquette une fois, puis se tait.
 narrateur|Victorina pose le carton contre l'épaule.
 narrateur|Une assiette tinte, puis se tait.
-narrateur|Le couloir laisse un rai, mince.</t>
+narrateur|Un rai mince dort dans le verre de la lampe.</t>
         </is>
       </c>
       <c r="AX69" t="inlineStr">
@@ -14141,17 +14141,17 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>Contre la chaise, le loup tient, dans le rond. On s'est assises, lampe au sol. Le haut gardera son ombre. Tiens bien le carton. La lampe ronde cliquette une fois, puis se tait. Victorina tapote le bois, léger. Une poussière s'envole, puis retombe. Une horloge tape, puis le buffet se tait.</t>
+          <t>Contre la chaise, le loup tient, dans le rond. On s'est assises, lampe au sol. Le haut gardera son ombre. Tiens bien le carton. La lampe ronde cliquette une fois, puis se tait. Victorina tapote le bois, léger. Une poussière s'envole, puis retombe. L'horloge tape, le rond se tait.</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Contre la chaise, le &lt;emphasis level="moderate"&gt;loup&lt;/emphasis&gt; tient, dans le rond. On s'est assises, lampe au sol. Le haut gardera son ombre. Tiens bien le carton. La lampe ronde cliquette une fois, puis se tait. Victorina tapote le bois, léger. Une poussière s'envole, puis retombe. Une horloge tape, puis le buffet se tait.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Contre la chaise, le &lt;emphasis level="moderate"&gt;loup&lt;/emphasis&gt; tient, dans le rond. On s'est assises, lampe au sol. Le haut gardera son ombre. Tiens bien le carton. La lampe ronde cliquette une fois, puis se tait. Victorina tapote le bois, léger. Une poussière s'envole, puis retombe. L'horloge tape, le rond se tait.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Contre la chaise, le &lt;emphasis&gt;loup&lt;/emphasis&gt; tient, dans le rond. On s'est assises, lampe au sol. Le haut gardera son ombre. Tiens bien le carton. La lampe ronde cliquette une fois, puis se tait. Victorina tapote le bois, léger. Une poussière s'envole, puis retombe. Une horloge tape, puis le buffet se tait.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Contre la chaise, le &lt;emphasis&gt;loup&lt;/emphasis&gt; tient, dans le rond. On s'est assises, lampe au sol. Le haut gardera son ombre. Tiens bien le carton. La lampe ronde cliquette une fois, puis se tait. Victorina tapote le bois, léger. Une poussière s'envole, puis retombe. L'horloge tape, le rond se tait.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr"/>
@@ -14296,7 +14296,7 @@
 narrateur|La lampe ronde cliquette une fois, puis se tait.
 narrateur|Victorina tapote le bois, léger.
 narrateur|Une poussière s'envole, puis retombe.
-narrateur|Une horloge tape, puis le buffet se tait.</t>
+narrateur|L'horloge tape, le rond se tait.</t>
         </is>
       </c>
       <c r="AX71" t="inlineStr">
@@ -14897,17 +14897,17 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>Loin de l'écho, la lune était là, dans le rond. Tu as fini, papa. Oui, le mot était long. Tu as tenu la porte. La lampe ronde cliquette une fois, puis se tait. Une poussière sèche sur le verre. Victorina fait marcher le loup, près du bois. Le placard redevient un placard, simple.</t>
+          <t>Loin de l'écho, la lune était là, dans le rond. Tu as fini, papa. Oui, le mot était long. Tu as tenu la porte. La lampe ronde cliquette une fois, puis se tait. Une poussière sèche sur le verre. Victorina fait marcher le loup, près du bois. Le verre de la lampe redevient froid.</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Loin de l'écho, la lune était là, dans le rond. Tu as fini, papa. Oui, le mot était long. Tu as tenu la porte. La lampe ronde cliquette une fois, puis se tait. Une poussière sèche sur le verre. Victorina fait marcher le &lt;emphasis level="moderate"&gt;loup&lt;/emphasis&gt;, près du bois. Le placard redevient un placard, simple.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Loin de l'écho, la lune était là, dans le rond. Tu as fini, papa. Oui, le mot était long. Tu as tenu la porte. La lampe ronde cliquette une fois, puis se tait. Une poussière sèche sur le verre. Victorina fait marcher le &lt;emphasis level="moderate"&gt;loup&lt;/emphasis&gt;, près du bois. Le verre de la lampe redevient froid.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Loin de l'écho, la lune était là, dans le rond. Tu as fini, papa. Oui, le mot était long. Tu as tenu la porte. La lampe ronde cliquette une fois, puis se tait. Une poussière sèche sur le verre. Victorina fait marcher le &lt;emphasis&gt;loup&lt;/emphasis&gt;, près du bois. Le placard redevient un placard, simple.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Loin de l'écho, la lune était là, dans le rond. Tu as fini, papa. Oui, le mot était long. Tu as tenu la porte. La lampe ronde cliquette une fois, puis se tait. Une poussière sèche sur le verre. Victorina fait marcher le &lt;emphasis&gt;loup&lt;/emphasis&gt;, près du bois. Le verre de la lampe redevient froid.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr"/>
@@ -15052,7 +15052,7 @@
 narrateur|La lampe ronde cliquette une fois, puis se tait.
 narrateur|Une poussière sèche sur le verre.
 narrateur|Victorina fait marcher le loup, près du bois.
-narrateur|Le placard redevient un placard, simple.</t>
+narrateur|Le verre de la lampe redevient froid.</t>
         </is>
       </c>
       <c r="AX75" t="inlineStr">
@@ -15084,17 +15084,17 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>Tout bas, sans le clic. Tout près des oreilles. L'écho recule, et le rond reste tiède. Derrière. Victorina souffle sur le verre, sans parler. Derrière la boîte. La lampe ronde dort contre sa paume. On a chuchoté ensemble. La suite a eu sa place.</t>
+          <t>Tout bas, sans le clic. Tout près des oreilles. L'écho recule, et le rond reste tiède. Derrière. Victorina souffle sur le verre, sans parler. Derrière la boîte. La lampe ronde dort contre sa paume. On a chuchoté ensemble. On l'entend, maintenant.</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Tout bas, sans le clic. Tout près des oreilles. L'écho recule, et le rond reste tiède. Derrière. Victorina souffle sur le verre, sans parler. Derrière la boîte. La lampe ronde dort contre sa paume. On a chuchoté ensemble. La suite a eu sa place.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Tout bas, sans le clic. Tout près des oreilles. L'écho recule, et le rond reste tiède. Derrière. Victorina souffle sur le verre, sans parler. Derrière la boîte. La lampe ronde dort contre sa paume. On a chuchoté ensemble. On l'entend, maintenant.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>Tout bas, sans le clic. Tout près des oreilles. L'écho recule, et le rond reste tiède. Derrière. Victorina souffle sur le verre, sans parler. Derrière la boîte. La lampe ronde dort contre sa paume. On a chuchoté ensemble. La suite a eu sa place. [pause]</t>
+          <t>Tout bas, sans le clic. Tout près des oreilles. L'écho recule, et le rond reste tiède. Derrière. Victorina souffle sur le verre, sans parler. Derrière la boîte. La lampe ronde dort contre sa paume. On a chuchoté ensemble. On l'entend, maintenant. [pause]</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr"/>
@@ -15236,7 +15236,7 @@
 maman|Derrière la boîte.
 narrateur|La lampe ronde dort contre sa paume.
 papa|On a chuchoté ensemble.
-maman|La suite a eu sa place.</t>
+maman|On l'entend, maintenant.</t>
         </is>
       </c>
       <c r="AX76" t="inlineStr">
@@ -15268,17 +15268,17 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>Dans le chuchotement, le rond a parlé. J'ai écouté, sans le clic. Tes oreilles étaient à la bonne place. Le mur t'attend. La lampe ronde cliquette une fois, puis se tait. Victorina essuie le verre sur son pantalon. Une ombre ronde reste sur le bois. Le loup avance, pas après pas.</t>
+          <t>Dans le chuchotement, le rond a parlé. J'ai écouté, sans le clic. Tes oreilles étaient à la bonne place. Le mur t'attend. La lampe ronde cliquette une fois, puis se tait. Victorina essuie le verre sur son pantalon. Le clic dort dans sa poche, oublié. Une ombre ronde reste collée au bois.</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Dans le chuchotement, le rond a parlé. J'ai écouté, sans le clic. Tes oreilles étaient à la bonne place. Le mur t'attend. La lampe ronde cliquette une fois, puis se tait. Victorina essuie le verre sur son pantalon. Une ombre ronde reste sur le bois. Le &lt;emphasis level="moderate"&gt;loup&lt;/emphasis&gt; avance, pas après pas.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Dans le chuchotement, le rond a parlé. J'ai écouté, sans le clic. Tes oreilles étaient à la bonne place. Le mur t'attend. La lampe ronde cliquette une fois, puis se tait. Victorina essuie le verre sur son pantalon. Le clic dort dans sa poche, oublié. Une ombre ronde reste collée au bois.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Dans le chuchotement, le rond a parlé. J'ai écouté, sans le clic. Tes oreilles étaient à la bonne place. Le mur t'attend. La lampe ronde cliquette une fois, puis se tait. Victorina essuie le verre sur son pantalon. Une ombre ronde reste sur le bois. Le &lt;emphasis&gt;loup&lt;/emphasis&gt; avance, pas après pas.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Dans le chuchotement, le rond a parlé. J'ai écouté, sans le clic. Tes oreilles étaient à la bonne place. Le mur t'attend. La lampe ronde cliquette une fois, puis se tait. Victorina essuie le verre sur son pantalon. Le clic dort dans sa poche, oublié. Une ombre ronde reste collée au bois.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr"/>
@@ -15422,8 +15422,8 @@
 maman|Le mur t'attend.
 narrateur|La lampe ronde cliquette une fois, puis se tait.
 narrateur|Victorina essuie le verre sur son pantalon.
-narrateur|Une ombre ronde reste sur le bois.
-narrateur|Le loup avance, pas après pas.</t>
+narrateur|Le clic dort dans sa poche, oublié.
+narrateur|Une ombre ronde reste collée au bois.</t>
         </is>
       </c>
       <c r="AX77" t="inlineStr">
@@ -15639,17 +15639,17 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>Sur la marche, la lune penche dans le rond. Je l'ai vue, contre le fond. Le bois a gardé l'ombre. Rentre le carton, après le pas. La lampe ronde cliquette une fois, puis se tait. Victorina souffle un peu sur les oreilles. Une poussière s'envole, puis retombe. La marche garde son ombre, seule.</t>
+          <t>Sur la marche, la lune penche dans le rond. Je l'ai vue, contre le fond. Le bois a gardé l'ombre. Rentre le carton, après le pas. La lampe ronde cliquette une fois, puis se tait. Victorina souffle un peu sur les oreilles. Une poussière s'envole, puis retombe. La marche garde un rond, puis l'oublie.</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Sur la marche, la lune penche dans le rond. Je l'ai vue, contre le fond. Le bois a gardé l'ombre. Rentre le carton, après le pas. La lampe ronde cliquette une fois, puis se tait. Victorina souffle un peu sur les oreilles. Une poussière s'envole, puis retombe. La marche garde son ombre, seule.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Sur la marche, la lune penche dans le rond. Je l'ai vue, contre le fond. Le bois a gardé l'ombre. Rentre le carton, après le pas. La lampe ronde cliquette une fois, puis se tait. Victorina souffle un peu sur les oreilles. Une poussière s'envole, puis retombe. La marche garde un rond, puis l'oublie.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Sur la marche, la lune penche dans le rond. Je l'ai vue, contre le fond. Le bois a gardé l'ombre. Rentre le carton, après le pas. La lampe ronde cliquette une fois, puis se tait. Victorina souffle un peu sur les oreilles. Une poussière s'envole, puis retombe. La marche garde son ombre, seule.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Sur la marche, la lune penche dans le rond. Je l'ai vue, contre le fond. Le bois a gardé l'ombre. Rentre le carton, après le pas. La lampe ronde cliquette une fois, puis se tait. Victorina souffle un peu sur les oreilles. Une poussière s'envole, puis retombe. La marche garde un rond, puis l'oublie.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr"/>
@@ -15794,7 +15794,7 @@
 narrateur|La lampe ronde cliquette une fois, puis se tait.
 narrateur|Victorina souffle un peu sur les oreilles.
 narrateur|Une poussière s'envole, puis retombe.
-narrateur|La marche garde son ombre, seule.</t>
+narrateur|La marche garde un rond, puis l'oublie.</t>
         </is>
       </c>
       <c r="AX79" t="inlineStr">
@@ -16395,17 +16395,17 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>Sur le tabouret, le rond a vu le cadre. Le mot est monté avec la lumière. Je remporte le tabouret, tout à l'heure. Essuie tes chaussettes, Victorina. La lampe ronde cliquette une fois, puis se tait. Le loup marche jusqu'au palier, dans le rond. Une marche se tait, puis l'autre. L'étagère redevient calme, une planche.</t>
+          <t>Sur le tabouret, le rond a vu le cadre. Le mot est monté avec la lumière. Je remporte le tabouret, tout à l'heure. Essuie tes chaussettes, Victorina. La lampe ronde cliquette une fois, puis se tait. Le loup marche jusqu'au palier, dans le rond. Une marche se tait, puis l'autre. Le palier garde un cercle, puis s'éteint.</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Sur le tabouret, le rond a vu le cadre. Le mot est monté avec la lumière. Je remporte le tabouret, tout à l'heure. Essuie tes chaussettes, Victorina. La lampe ronde cliquette une fois, puis se tait. Le &lt;emphasis level="moderate"&gt;loup&lt;/emphasis&gt; marche jusqu'au palier, dans le rond. Une marche se tait, puis l'autre. L'étagère redevient calme, une planche.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Sur le tabouret, le rond a vu le cadre. Le mot est monté avec la lumière. Je remporte le tabouret, tout à l'heure. Essuie tes chaussettes, Victorina. La lampe ronde cliquette une fois, puis se tait. Le &lt;emphasis level="moderate"&gt;loup&lt;/emphasis&gt; marche jusqu'au palier, dans le rond. Une marche se tait, puis l'autre. Le palier garde un cercle, puis s'éteint.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Sur le tabouret, le rond a vu le cadre. Le mot est monté avec la lumière. Je remporte le tabouret, tout à l'heure. Essuie tes chaussettes, Victorina. La lampe ronde cliquette une fois, puis se tait. Le &lt;emphasis&gt;loup&lt;/emphasis&gt; marche jusqu'au palier, dans le rond. Une marche se tait, puis l'autre. L'étagère redevient calme, une planche.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Sur le tabouret, le rond a vu le cadre. Le mot est monté avec la lumière. Je remporte le tabouret, tout à l'heure. Essuie tes chaussettes, Victorina. La lampe ronde cliquette une fois, puis se tait. Le &lt;emphasis&gt;loup&lt;/emphasis&gt; marche jusqu'au palier, dans le rond. Une marche se tait, puis l'autre. Le palier garde un cercle, puis s'éteint.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr"/>
@@ -16550,7 +16550,7 @@
 narrateur|La lampe ronde cliquette une fois, puis se tait.
 narrateur|Le loup marche jusqu'au palier, dans le rond.
 narrateur|Une marche se tait, puis l'autre.
-narrateur|L'étagère redevient calme, une planche.</t>
+narrateur|Le palier garde un cercle, puis s'éteint.</t>
         </is>
       </c>
       <c r="AX83" t="inlineStr">
@@ -16582,17 +16582,17 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>Le rond regarde en bas. Victorina baisse la lampe, vers la plinthe. Pas le grand. Le petit, contre le bois. Une lune de papier penche, bas, tombée. Le rond la réveille, sans un clic. La lampe ronde dort contre sa paume. Le mot a fini sa route. Merci d'avoir regardé jusque-là.</t>
+          <t>Le rond regarde en bas. Victorina baisse la lampe, vers la plinthe. Pas le grand. Le petit, contre le bois. Une lune de papier penche, bas, tombée. Le rond la réveille, sans un clic. La lampe ronde dort contre sa paume. Elle attendait là, tout bas. Merci d'avoir baissé les yeux.</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le rond regarde en bas. Victorina baisse la lampe, vers la &lt;emphasis level="moderate"&gt;plinthe&lt;/emphasis&gt;. Pas le grand. Le petit, contre le bois. Une lune de papier penche, bas, tombée. Le rond la réveille, sans un clic. La lampe ronde dort contre sa paume. Le mot a fini sa route. Merci d'avoir regardé jusque-là.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le rond regarde en bas. Victorina baisse la lampe, vers la &lt;emphasis level="moderate"&gt;plinthe&lt;/emphasis&gt;. Pas le grand. Le petit, contre le bois. Une lune de papier penche, bas, tombée. Le rond la réveille, sans un clic. La lampe ronde dort contre sa paume. Elle attendait là, tout bas. Merci d'avoir baissé les yeux.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>Le rond regarde en bas. Victorina baisse la lampe, vers la &lt;emphasis&gt;plinthe&lt;/emphasis&gt;. Pas le grand. Le petit, contre le bois. Une lune de papier penche, bas, tombée. Le rond la réveille, sans un clic. La lampe ronde dort contre sa paume. Le mot a fini sa route. Merci d'avoir regardé jusque-là. [pause]</t>
+          <t>Le rond regarde en bas. Victorina baisse la lampe, vers la &lt;emphasis&gt;plinthe&lt;/emphasis&gt;. Pas le grand. Le petit, contre le bois. Une lune de papier penche, bas, tombée. Le rond la réveille, sans un clic. La lampe ronde dort contre sa paume. Elle attendait là, tout bas. Merci d'avoir baissé les yeux. [pause]</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr"/>
@@ -16733,8 +16733,8 @@
 narrateur|Une lune de papier penche, bas, tombée.
 narrateur|Le rond la réveille, sans un clic.
 narrateur|La lampe ronde dort contre sa paume.
-maman|Le mot a fini sa route.
-papa|Merci d'avoir regardé jusque-là.</t>
+maman|Elle attendait là, tout bas.
+papa|Merci d'avoir baissé les yeux.</t>
         </is>
       </c>
       <c r="AX84" t="inlineStr">
@@ -16766,17 +16766,17 @@
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>Tout en bas, la lune brille dans le rond, près de la plinthe. Tu as dit petit, à la fin. Merci d'avoir écouté jusque-là. Un peu de lait, après le mur. La lampe ronde cliquette une fois, puis se tait. Victorina pose le carton contre le mur du palier. L'étagère reprend sa place, sage. Le haut n'a plus de secret, ce soir.</t>
+          <t>Tout en bas, la lune brille dans le rond, près de la plinthe. Tu as dit petit, à la fin. Merci d'avoir regardé en bas. Le savon t'attend, près de l'eau. La lampe ronde cliquette une fois, puis se tait. Victorina pose le carton contre le mur du palier. L'étagère reprend sa place, sage. La plinthe reprend son ombre, sans secret.</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Tout en bas, la lune brille dans le rond, près de la plinthe. Tu as dit petit, à la fin. Merci d'avoir écouté jusque-là. Un peu de lait, après le mur. La lampe ronde cliquette une fois, puis se tait. Victorina pose le carton contre le mur du palier. L'étagère reprend sa place, sage. Le haut n'a plus de secret, ce soir.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Tout en bas, la lune brille dans le rond, près de la plinthe. Tu as dit petit, à la fin. Merci d'avoir regardé en bas. Le savon t'attend, près de l'eau. La lampe ronde cliquette une fois, puis se tait. Victorina pose le carton contre le mur du palier. L'étagère reprend sa place, sage. La plinthe reprend son ombre, sans secret.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Tout en bas, la lune brille dans le rond, près de la plinthe. Tu as dit petit, à la fin. Merci d'avoir écouté jusque-là. Un peu de lait, après le mur. La lampe ronde cliquette une fois, puis se tait. Victorina pose le carton contre le mur du palier. L'étagère reprend sa place, sage. Le haut n'a plus de secret, ce soir.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Tout en bas, la lune brille dans le rond, près de la plinthe. Tu as dit petit, à la fin. Merci d'avoir regardé en bas. Le savon t'attend, près de l'eau. La lampe ronde cliquette une fois, puis se tait. Victorina pose le carton contre le mur du palier. L'étagère reprend sa place, sage. La plinthe reprend son ombre, sans secret.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr"/>
@@ -16916,12 +16916,12 @@
         <is>
           <t>narrateur|Tout en bas, la lune brille dans le rond, près de la plinthe.
 enfant-f|Tu as dit petit, à la fin.
-papa|Merci d'avoir écouté jusque-là.
-maman|Un peu de lait, après le mur.
+papa|Merci d'avoir regardé en bas.
+maman|Le savon t'attend, près de l'eau.
 narrateur|La lampe ronde cliquette une fois, puis se tait.
 narrateur|Victorina pose le carton contre le mur du palier.
 narrateur|L'étagère reprend sa place, sage.
-narrateur|Le haut n'a plus de secret, ce soir.</t>
+narrateur|La plinthe reprend son ombre, sans secret.</t>
         </is>
       </c>
       <c r="AX85" t="inlineStr">
@@ -16953,17 +16953,17 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>Tes bras, et la lampe. Viens, tout contre moi. Victorina s'élève, le rond entre les livres. La lune, tout près du bord. Le rond l'a eue ! Un rond blanc brille entre deux livres, enfin. La lampe ronde dort contre sa paume. Tes bras ont fini la phrase. Chacun a fait sa part.</t>
+          <t>Tes bras, et la lampe. Viens, tout contre moi. Victorina s'élève, le rond entre les livres. La lune, tout près du bord. Le rond l'a eue ! Un rond blanc brille entre deux livres, enfin. La lampe ronde dort contre sa paume. Elle est entre les livres. Chacun a fait sa part.</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Tes &lt;emphasis level="moderate"&gt;bras&lt;/emphasis&gt;, et la lampe. Viens, tout contre moi. Victorina s'élève, le rond entre les livres. La lune, tout près du bord. Le rond l'a eue ! Un rond blanc brille entre deux livres, enfin. La lampe ronde dort contre sa paume. Tes bras ont fini la phrase. Chacun a fait sa part.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Tes &lt;emphasis level="moderate"&gt;bras&lt;/emphasis&gt;, et la lampe. Viens, tout contre moi. Victorina s'élève, le rond entre les livres. La lune, tout près du bord. Le rond l'a eue ! Un rond blanc brille entre deux livres, enfin. La lampe ronde dort contre sa paume. Elle est entre les livres. Chacun a fait sa part.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>Tes &lt;emphasis&gt;bras&lt;/emphasis&gt;, et la lampe. Viens, tout contre moi. Victorina s'élève, le rond entre les livres. La lune, tout près du bord. Le rond l'a eue ! Un rond blanc brille entre deux livres, enfin. La lampe ronde dort contre sa paume. Tes bras ont fini la phrase. Chacun a fait sa part. [pause]</t>
+          <t>Tes &lt;emphasis&gt;bras&lt;/emphasis&gt;, et la lampe. Viens, tout contre moi. Victorina s'élève, le rond entre les livres. La lune, tout près du bord. Le rond l'a eue ! Un rond blanc brille entre deux livres, enfin. La lampe ronde dort contre sa paume. Elle est entre les livres. Chacun a fait sa part. [pause]</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr"/>
@@ -17104,7 +17104,7 @@
 enfant-f|Le rond l'a eue !
 narrateur|Un rond blanc brille entre deux livres, enfin.
 narrateur|La lampe ronde dort contre sa paume.
-maman|Tes bras ont fini la phrase.
+maman|Elle est entre les livres.
 papa|Chacun a fait sa part.</t>
         </is>
       </c>
@@ -17137,17 +17137,17 @@
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>Dans les bras de papa, le rond a pris la lune. On l'a prise, tout haut. Tes yeux allaient assez loin. Le haut gardera son ombre. La lampe ronde cliquette une fois, puis se tait. Victorina pose le carton près des carreaux. Les oreilles touchent l'air. Une bande jaune s'allonge, puis la lampe se tait.</t>
+          <t>Dans les bras de papa, le rond a pris la lune. On l'a prise, tout haut. Tes yeux allaient assez loin. Le haut gardera son ombre. La lampe ronde cliquette une fois, puis se tait. Victorina pose le carton près des carreaux. Les oreilles touchent l'air. La bande jaune s'allonge, et le rond s'éteint.</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Dans les bras de papa, le rond a pris la lune. On l'a prise, tout haut. Tes yeux allaient assez loin. Le haut gardera son ombre. La lampe ronde cliquette une fois, puis se tait. Victorina pose le carton près des carreaux. Les oreilles touchent l'air. Une bande jaune s'allonge, puis la lampe se tait.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Dans les bras de papa, le rond a pris la lune. On l'a prise, tout haut. Tes yeux allaient assez loin. Le haut gardera son ombre. La lampe ronde cliquette une fois, puis se tait. Victorina pose le carton près des carreaux. Les oreilles touchent l'air. La bande jaune s'allonge, et le rond s'éteint.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Dans les bras de papa, le rond a pris la lune. On l'a prise, tout haut. Tes yeux allaient assez loin. Le haut gardera son ombre. La lampe ronde cliquette une fois, puis se tait. Victorina pose le carton près des carreaux. Les oreilles touchent l'air. Une bande jaune s'allonge, puis la lampe se tait.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Dans les bras de papa, le rond a pris la lune. On l'a prise, tout haut. Tes yeux allaient assez loin. Le haut gardera son ombre. La lampe ronde cliquette une fois, puis se tait. Victorina pose le carton près des carreaux. Les oreilles touchent l'air. La bande jaune s'allonge, et le rond s'éteint.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr"/>
@@ -17292,7 +17292,7 @@
 narrateur|La lampe ronde cliquette une fois, puis se tait.
 narrateur|Victorina pose le carton près des carreaux.
 narrateur|Les oreilles touchent l'air.
-narrateur|Une bande jaune s'allonge, puis la lampe se tait.</t>
+narrateur|La bande jaune s'allonge, et le rond s'éteint.</t>
         </is>
       </c>
       <c r="AX87" t="inlineStr">
@@ -17318,7 +17318,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17424,6 +17424,13 @@
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>